<commit_message>
UAT Round 3 — fix 22 remaining issues
Root causes found and fixed:
- #7: SMS handler now handles booking.confirmed event type
- #10: Booking spot link shows "View listing" fallback when address empty
- #14/#49: Photo extraction handles both string and object formats
- #18-21: Cancel button hidden for ACTIVE bookings
- #4: Chat partner fetched from /users/{id}/public (was /profile)
- #26: CallToAction hidden when user logged in
- #12/#13: ModifyModal receives booking status + dynamic pricePerHour
- #36: Invoicing saved to sessionStorage on Continue click
- #5: Chat container height calc(100vh - 72px), flex message area
- #30: Card aspect ratio 1/2.1 for more vertical space

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documentation/Issue-tracker-spotzy.xlsx
+++ b/documentation/Issue-tracker-spotzy.xlsx
@@ -8,14 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/orfeopreto/Dev/Claude/spotzy/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA64778C-B9E8-3F48-B734-7F47A1576655}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2A3C5EF-419A-4D48-85F3-5B7606C16A4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-2420" yWindow="-21600" windowWidth="38400" windowHeight="21600" xr2:uid="{EF712131-2427-7943-B2E8-AD061EC4DE1A}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="1" xr2:uid="{EF712131-2427-7943-B2E8-AD061EC4DE1A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1 (2)" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sheet1 (2)'!$A$1:$G$53</definedName>
+  </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -37,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="149">
   <si>
     <t>Host Dashboard</t>
   </si>
@@ -349,9 +352,6 @@
   </si>
   <si>
     <t>don't add country prefix to phone number textbox but concatenate on submit. Remove leading 0 from value phone textbox</t>
-  </si>
-  <si>
-    <t>link</t>
   </si>
   <si>
     <t>Intake invoicing data on account page, cannot submit edited content</t>
@@ -437,12 +437,6 @@
     <t>linked to</t>
   </si>
   <si>
-    <t>when clicking on link to listing redirected to landing page</t>
-  </si>
-  <si>
-    <t>redirect to listing</t>
-  </si>
-  <si>
     <t xml:space="preserve">Host dashboard </t>
   </si>
   <si>
@@ -453,9 +447,6 @@
   </si>
   <si>
     <t>landing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  dynamically resized</t>
   </si>
   <si>
     <t xml:space="preserve">tooltip size is hardcoded
@@ -463,16 +454,61 @@
   </si>
   <si>
     <t>move bounds of tooltip so that it can appear on the map</t>
+  </si>
+  <si>
+    <t>public profile page doesn't load; cilent side error:
+e.photos[0].startsWith is not a function</t>
+  </si>
+  <si>
+    <t>should load and show images</t>
+  </si>
+  <si>
+    <t>/users/…</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  dynamically resized based on map size and zoom</t>
+  </si>
+  <si>
+    <t>when clicking on link edit listing redirected to landing page</t>
+  </si>
+  <si>
+    <t>redirect to listing edit page</t>
+  </si>
+  <si>
+    <t>chat window height is 20% but the container size is still too big</t>
+  </si>
+  <si>
+    <t>cointainer of chat window must be resized too (20% of screen height)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CTA "create account" under "Ready to find your spot"  is visible even when logged on </t>
+  </si>
+  <si>
+    <t xml:space="preserve">shold not be visible if user is logged on </t>
+  </si>
+  <si>
+    <t>can't see bot responses in previous conversations</t>
+  </si>
+  <si>
+    <t>should see all messages in previous conversation</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="0"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -500,7 +536,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -513,13 +549,34 @@
         <bgColor theme="0" tint="-0.14999847407452621"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor theme="1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="medium">
+        <color theme="1"/>
+      </top>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -567,78 +624,57 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <b/>
@@ -679,7 +715,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{86F359F2-41C3-D443-B0FE-5E6EB3FE039F}" name="Table2" displayName="Table2" ref="A1:G34" totalsRowShown="0" headerRowDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{86F359F2-41C3-D443-B0FE-5E6EB3FE039F}" name="Table2" displayName="Table2" ref="A1:G34" totalsRowShown="0" headerRowDxfId="0">
   <autoFilter ref="A1:G34" xr:uid="{86F359F2-41C3-D443-B0FE-5E6EB3FE039F}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F34">
     <sortCondition ref="E1:E34"/>
@@ -689,25 +725,9 @@
     <tableColumn id="2" xr3:uid="{B88367C6-293B-EE43-9A65-44CD4F8A6890}" name="pro-condition / action"/>
     <tableColumn id="3" xr3:uid="{F5672D69-4329-674E-8270-36C224EBB500}" name="observed behaviour"/>
     <tableColumn id="4" xr3:uid="{D69BD67C-D8A0-ED4A-A02F-B2A10159DE64}" name="expected behaviour"/>
-    <tableColumn id="5" xr3:uid="{165D054A-4C73-DE48-A9D4-05EB5A97FC62}" name="page" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{165D054A-4C73-DE48-A9D4-05EB5A97FC62}" name="page" dataDxfId="1"/>
     <tableColumn id="6" xr3:uid="{B5946274-981C-DE41-A836-680968ABEA8F}" name="2nd test passed"/>
     <tableColumn id="7" xr3:uid="{63425FD8-6197-5E45-A845-3A5B03F9FB02}" name="linked to"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1FBCA233-C12E-704C-ABE5-94346D4A305E}" name="Table24" displayName="Table24" ref="A1:G12" totalsRowShown="0" headerRowDxfId="2">
-  <autoFilter ref="A1:G12" xr:uid="{86F359F2-41C3-D443-B0FE-5E6EB3FE039F}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{FA329104-AC39-9C44-8C5B-FD95363C9EA5}" name="Number"/>
-    <tableColumn id="2" xr3:uid="{D6167578-3E36-554C-88BD-B6C67546CE6F}" name="pro-condition / action"/>
-    <tableColumn id="3" xr3:uid="{1ACF5FC4-ED6F-B946-A744-F991E74B6F2E}" name="observed behaviour" dataDxfId="0"/>
-    <tableColumn id="4" xr3:uid="{EA610275-215E-E845-A069-38009596233F}" name="expected behaviour"/>
-    <tableColumn id="5" xr3:uid="{AADDEE1A-E2BA-9F49-9F74-3E82D85559C8}" name="page" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{70AD95F3-76F2-6445-8352-9CE0C35AEF3C}" name="2nd test passed"/>
-    <tableColumn id="7" xr3:uid="{D930F407-F360-1E44-A12C-8325627CBE78}" name="link"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1030,7 +1050,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{922DD406-F819-574C-B490-24B3D9D05D6D}">
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="39.33203125" customWidth="1"/>
@@ -1056,11 +1076,11 @@
       <c r="E1" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="10" t="s">
         <v>97</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -1080,7 +1100,7 @@
         <v>23</v>
       </c>
       <c r="F2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -1134,7 +1154,7 @@
         <v>16</v>
       </c>
       <c r="F5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -1162,7 +1182,7 @@
         <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C7" t="s">
         <v>59</v>
@@ -1262,7 +1282,7 @@
         <v>9</v>
       </c>
       <c r="F12" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -1282,7 +1302,7 @@
         <v>29</v>
       </c>
       <c r="F13" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -1299,7 +1319,7 @@
         <v>0</v>
       </c>
       <c r="F14" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -1316,7 +1336,7 @@
         <v>0</v>
       </c>
       <c r="F15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -1333,7 +1353,7 @@
         <v>0</v>
       </c>
       <c r="F16" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -1367,7 +1387,7 @@
         <v>0</v>
       </c>
       <c r="F18" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
@@ -1404,7 +1424,7 @@
         <v>73</v>
       </c>
       <c r="F20" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
@@ -1478,7 +1498,7 @@
         <v>70</v>
       </c>
       <c r="F24" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
@@ -1495,7 +1515,7 @@
         <v>61</v>
       </c>
       <c r="F25" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
@@ -1546,7 +1566,7 @@
         <v>39</v>
       </c>
       <c r="F28" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
@@ -1563,7 +1583,7 @@
         <v>14</v>
       </c>
       <c r="F29" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
@@ -1583,7 +1603,7 @@
         <v>14</v>
       </c>
       <c r="F30" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
@@ -1623,7 +1643,7 @@
         <v>46</v>
       </c>
       <c r="F32" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
@@ -1643,7 +1663,7 @@
         <v>46</v>
       </c>
       <c r="F33" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -1667,302 +1687,325 @@
       </c>
     </row>
     <row r="35" spans="1:7" ht="51" x14ac:dyDescent="0.2">
-      <c r="A35" s="6">
+      <c r="A35" s="7">
         <v>34</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="B35" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="C35" s="11" t="s">
+      <c r="C35" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="D35" s="6" t="s">
+      <c r="D35" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="E35" s="6" t="s">
+      <c r="E35" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="F35" s="6" t="s">
+      <c r="F35" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="G35" s="7"/>
+    </row>
+    <row r="36" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A36" s="8">
+        <v>35</v>
+      </c>
+      <c r="B36" s="8"/>
+      <c r="C36" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="D36" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="E36" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="G36" s="8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A37" s="7">
+        <v>36</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="C37" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="E37" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="F37" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="G37" s="7">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A38" s="8">
+        <v>37</v>
+      </c>
+      <c r="B38" s="8"/>
+      <c r="C38" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="D38" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="G35" s="6"/>
-    </row>
-    <row r="36" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A36" s="7">
-        <v>35</v>
-      </c>
-      <c r="B36" s="7"/>
-      <c r="C36" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="D36" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="E36" s="7" t="s">
+      <c r="E38" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="F36" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="G36" s="7">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A37" s="6">
-        <v>36</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="C37" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="D37" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="E37" s="13" t="s">
-        <v>100</v>
-      </c>
-      <c r="F37" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="G37" s="6">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A38" s="7">
-        <v>37</v>
-      </c>
-      <c r="B38" s="7"/>
-      <c r="C38" s="12" t="s">
+      <c r="F38" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="G38" s="8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A39" s="7">
+        <v>38</v>
+      </c>
+      <c r="B39" s="7"/>
+      <c r="C39" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="D39" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="D38" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="E38" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="F38" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="G38" s="7">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A39" s="6">
-        <v>38</v>
-      </c>
-      <c r="B39" s="6"/>
-      <c r="C39" s="11" t="s">
+      <c r="E39" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="D39" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="E39" s="13" t="s">
+      <c r="F39" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="G39" s="7">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A40" s="8">
+        <v>39</v>
+      </c>
+      <c r="B40" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="F39" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="G39" s="6">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A40" s="7">
-        <v>39</v>
-      </c>
-      <c r="B40" s="12" t="s">
+      <c r="C40" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="C40" s="12" t="s">
+      <c r="D40" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="D40" s="7" t="s">
+      <c r="E40" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="E40" s="14" t="s">
+      <c r="F40" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="G40" s="8">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+      <c r="A41" s="7">
+        <v>40</v>
+      </c>
+      <c r="B41" s="12"/>
+      <c r="C41" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="F40" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="G40" s="7">
+      <c r="D41" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="E41" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="F41" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="G41" s="7">
         <v>13</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="68" x14ac:dyDescent="0.2">
-      <c r="A41" s="6">
-        <v>40</v>
-      </c>
-      <c r="B41" s="11"/>
-      <c r="C41" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="D41" s="11" t="s">
+    <row r="42" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A42" s="8">
+        <v>41</v>
+      </c>
+      <c r="B42" s="8"/>
+      <c r="C42" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="D42" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="E42" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="E41" s="13" t="s">
-        <v>116</v>
-      </c>
-      <c r="F41" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="G41" s="6">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A42" s="7">
-        <v>41</v>
-      </c>
-      <c r="B42" s="7"/>
-      <c r="C42" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="D42" s="7" t="s">
+      <c r="F42" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="G42" s="8"/>
+    </row>
+    <row r="43" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A43" s="7">
+        <v>42</v>
+      </c>
+      <c r="B43" s="7"/>
+      <c r="C43" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="E42" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="F42" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="G42" s="7"/>
-    </row>
-    <row r="43" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A43" s="6">
-        <v>42</v>
-      </c>
-      <c r="B43" s="6"/>
-      <c r="C43" s="11" t="s">
+      <c r="D43" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="D43" s="6" t="s">
+      <c r="E43" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="E43" s="13" t="s">
-        <v>124</v>
-      </c>
-      <c r="F43" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="G43" s="6"/>
+      <c r="F43" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="G43" s="7"/>
     </row>
     <row r="44" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A44" s="7">
+      <c r="A44" s="8">
         <v>43</v>
       </c>
-      <c r="B44" s="7" t="s">
+      <c r="B44" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="C44" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="C44" s="12" t="s">
+      <c r="D44" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="D44" s="12" t="s">
-        <v>130</v>
-      </c>
-      <c r="E44" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="F44" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="G44" s="7"/>
+      <c r="E44" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="F44" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="G44" s="8"/>
     </row>
     <row r="45" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="8">
+      <c r="A45" s="9">
         <v>44</v>
       </c>
-      <c r="B45" s="8"/>
-      <c r="C45" s="15" t="s">
+      <c r="B45" s="9"/>
+      <c r="C45" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="D45" s="8" t="s">
+      <c r="D45" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="E45" s="16" t="s">
-        <v>126</v>
-      </c>
-      <c r="F45" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="G45" s="8">
+      <c r="E45" s="17" t="s">
+        <v>125</v>
+      </c>
+      <c r="F45" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="G45" s="9">
         <v>25</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A46" s="17">
+      <c r="A46" s="18">
         <v>45</v>
       </c>
       <c r="C46" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="D46" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G46">
         <v>24</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A47" s="18">
+      <c r="A47" s="19">
         <v>46</v>
       </c>
       <c r="C47" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="D47" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>137</v>
+        <v>134</v>
+      </c>
+      <c r="F47" s="20" t="s">
+        <v>106</v>
       </c>
       <c r="G47">
         <v>44</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A48" s="17">
+      <c r="A48" s="18">
         <v>47</v>
       </c>
-      <c r="C48" s="10" t="s">
-        <v>139</v>
+      <c r="C48" s="11" t="s">
+        <v>135</v>
       </c>
       <c r="D48" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
+      </c>
+      <c r="F48" t="s">
+        <v>96</v>
       </c>
       <c r="G48">
         <v>43</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A49" s="17">
+    <row r="49" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A49" s="18">
         <v>48</v>
       </c>
-      <c r="C49" s="10" t="s">
-        <v>129</v>
+      <c r="C49" s="11" t="s">
+        <v>128</v>
       </c>
       <c r="D49" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
+      </c>
+      <c r="F49" t="s">
+        <v>106</v>
       </c>
       <c r="G49">
         <v>43</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A50" s="18">
+        <v>49</v>
+      </c>
+      <c r="C50" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="D50" t="s">
+        <v>138</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -1975,7 +2018,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2459A4F-4D1F-D947-9C74-71F227501814}">
-  <dimension ref="A1:G12"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="47.1640625" customWidth="1"/>
@@ -1985,221 +2029,1005 @@
     <col min="6" max="6" width="23.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>19</v>
+      </c>
+      <c r="B6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F6" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
+        <v>124</v>
+      </c>
+      <c r="C7" t="s">
+        <v>59</v>
+      </c>
+      <c r="D7" t="s">
+        <v>58</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>21</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>18</v>
+      </c>
+      <c r="C9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" t="s">
+        <v>51</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F9" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>4</v>
+      </c>
+      <c r="C10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F10" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>5</v>
+      </c>
+      <c r="C11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>8</v>
+      </c>
+      <c r="C12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F13" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>1</v>
+      </c>
+      <c r="D14" t="s">
+        <v>2</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F14" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>2</v>
+      </c>
+      <c r="C15" t="s">
+        <v>3</v>
+      </c>
+      <c r="D15" t="s">
+        <v>4</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F15" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>3</v>
+      </c>
+      <c r="C16" t="s">
+        <v>5</v>
+      </c>
+      <c r="D16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>23</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D17" t="s">
+        <v>65</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F17" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>24</v>
+      </c>
+      <c r="C18" t="s">
+        <v>66</v>
+      </c>
+      <c r="D18" t="s">
+        <v>67</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F18" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>26</v>
+      </c>
+      <c r="C19" t="s">
+        <v>71</v>
+      </c>
+      <c r="D19" t="s">
+        <v>72</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F19" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>27</v>
+      </c>
+      <c r="B20" t="s">
+        <v>76</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D20" t="s">
+        <v>74</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F20" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>15</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21" t="s">
+        <v>41</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F21" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>12</v>
+      </c>
+      <c r="B22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C22" t="s">
+        <v>31</v>
+      </c>
+      <c r="D22" t="s">
+        <v>32</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F22" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>13</v>
+      </c>
+      <c r="B23" t="s">
+        <v>34</v>
+      </c>
+      <c r="C23" t="s">
+        <v>35</v>
+      </c>
+      <c r="D23" t="s">
+        <v>36</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F23" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A24">
+        <v>25</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D24" t="s">
+        <v>69</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F24" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>22</v>
+      </c>
+      <c r="C25" t="s">
+        <v>62</v>
+      </c>
+      <c r="D25" t="s">
+        <v>63</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F25" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A26">
+        <v>14</v>
+      </c>
+      <c r="C26" t="s">
+        <v>37</v>
+      </c>
+      <c r="D26" t="s">
+        <v>38</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F26" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>31</v>
+      </c>
+      <c r="C27" t="s">
+        <v>84</v>
+      </c>
+      <c r="D27" t="s">
+        <v>85</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F27" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>32</v>
+      </c>
+      <c r="C28" t="s">
+        <v>86</v>
+      </c>
+      <c r="D28" t="s">
+        <v>87</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F28" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>6</v>
+      </c>
+      <c r="C29" t="s">
+        <v>12</v>
+      </c>
+      <c r="D29" t="s">
+        <v>13</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F29" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A30">
+        <v>33</v>
+      </c>
+      <c r="B30" t="s">
+        <v>88</v>
+      </c>
+      <c r="C30" t="s">
+        <v>90</v>
+      </c>
+      <c r="D30" t="s">
+        <v>89</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>16</v>
+      </c>
+      <c r="B31" t="s">
+        <v>43</v>
+      </c>
+      <c r="C31" t="s">
+        <v>45</v>
+      </c>
+      <c r="D31" t="s">
+        <v>44</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F31" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A32">
+        <v>28</v>
+      </c>
+      <c r="B32" t="s">
+        <v>77</v>
+      </c>
+      <c r="C32" t="s">
+        <v>78</v>
+      </c>
+      <c r="D32" t="s">
+        <v>79</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F32" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A33">
+        <v>29</v>
+      </c>
+      <c r="B33" t="s">
+        <v>77</v>
+      </c>
+      <c r="C33" t="s">
+        <v>80</v>
+      </c>
+      <c r="D33" t="s">
+        <v>81</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F33" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A34">
+        <v>30</v>
+      </c>
+      <c r="B34" t="s">
+        <v>77</v>
+      </c>
+      <c r="C34" t="s">
+        <v>82</v>
+      </c>
+      <c r="D34" t="s">
+        <v>83</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F34" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="51" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="7">
+        <v>34</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="G35" s="7"/>
+    </row>
+    <row r="36" spans="1:7" ht="34" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="8">
+        <v>35</v>
+      </c>
+      <c r="B36" s="8"/>
+      <c r="C36" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="D36" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="E36" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="G36" s="8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A37" s="7">
+        <v>36</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="C37" s="12" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" ht="51" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>34</v>
-      </c>
-      <c r="B2" t="s">
-        <v>98</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="D2" t="s">
-        <v>99</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="D37" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="E37" s="14" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A3">
-        <v>35</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="F37" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="G37" s="7">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A38" s="8">
+        <v>37</v>
+      </c>
+      <c r="B38" s="8"/>
+      <c r="C38" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="E38" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="G3">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A4">
-        <v>36</v>
-      </c>
-      <c r="B4" t="s">
-        <v>98</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="D4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="G4">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>37</v>
-      </c>
-      <c r="C5" s="10" t="s">
+      <c r="F38" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="G38" s="8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="34" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="7">
+        <v>38</v>
+      </c>
+      <c r="B39" s="7"/>
+      <c r="C39" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="D39" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="D5" t="s">
-        <v>108</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="G5">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>38</v>
-      </c>
-      <c r="C6" s="10" t="s">
+      <c r="E39" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="D6" t="s">
-        <v>110</v>
-      </c>
-      <c r="E6" s="1" t="s">
+      <c r="F39" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="G39" s="7">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="34" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="8">
+        <v>39</v>
+      </c>
+      <c r="B40" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="G6">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A7">
+      <c r="C40" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="D40" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="E40" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="F40" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="G40" s="8">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="68" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="7">
+        <v>40</v>
+      </c>
+      <c r="B41" s="12"/>
+      <c r="C41" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="D41" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="E41" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="F41" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="G41" s="7">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="34" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="8">
+        <v>41</v>
+      </c>
+      <c r="B42" s="8"/>
+      <c r="C42" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="D42" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="E42" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="F42" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="G42" s="8"/>
+    </row>
+    <row r="43" spans="1:7" ht="17" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="7">
+        <v>42</v>
+      </c>
+      <c r="B43" s="7"/>
+      <c r="C43" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="E43" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="G43" s="7"/>
+    </row>
+    <row r="44" spans="1:7" ht="34" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="8">
+        <v>43</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="C44" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="D44" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="E44" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="F44" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="G44" s="8"/>
+    </row>
+    <row r="45" spans="1:7" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="9">
+        <v>44</v>
+      </c>
+      <c r="B45" s="9"/>
+      <c r="C45" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="E45" s="17" t="s">
+        <v>125</v>
+      </c>
+      <c r="F45" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="G45" s="9">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A46" s="18">
+        <v>45</v>
+      </c>
+      <c r="C46" t="s">
+        <v>141</v>
+      </c>
+      <c r="D46" t="s">
+        <v>142</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="G46">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="19">
+        <v>46</v>
+      </c>
+      <c r="C47" t="s">
+        <v>132</v>
+      </c>
+      <c r="D47" t="s">
+        <v>133</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="F47" s="20" t="s">
+        <v>106</v>
+      </c>
+      <c r="G47">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A48" s="18">
+        <v>47</v>
+      </c>
+      <c r="C48" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="D48" t="s">
+        <v>140</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="F48" t="s">
+        <v>96</v>
+      </c>
+      <c r="G48">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" ht="34" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="18">
+        <v>48</v>
+      </c>
+      <c r="C49" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="D49" t="s">
+        <v>136</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="F49" t="s">
+        <v>106</v>
+      </c>
+      <c r="G49">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A50" s="18">
+        <v>49</v>
+      </c>
+      <c r="C50" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="D50" t="s">
+        <v>138</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="C51" s="22" t="s">
+        <v>143</v>
+      </c>
+      <c r="D51" t="s">
+        <v>144</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G51">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="C52" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="D52" t="s">
+        <v>146</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A53" s="8">
         <v>39</v>
       </c>
-      <c r="B7" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>114</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="B53" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="C53" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="D53" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="E53" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="G7">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="68" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>40</v>
-      </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="G8">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <v>41</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="D9" t="s">
-        <v>121</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A10">
-        <v>42</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>122</v>
-      </c>
-      <c r="D10" t="s">
-        <v>123</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A11">
-        <v>43</v>
-      </c>
-      <c r="B11" t="s">
-        <v>128</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12">
-        <v>44</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="D12" t="s">
-        <v>69</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="G12">
-        <v>25</v>
-      </c>
+      <c r="F53" s="8"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G53" xr:uid="{E2459A4F-4D1F-D947-9C74-71F227501814}">
+    <filterColumn colId="5">
+      <filters blank="1">
+        <filter val="no"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix 7 test regressions from UAT Round 3
- CancelModal tests: use future dates (2027) and time-tier-appropriate
  booking start times instead of past dates
- Dispute tests: add MSW handler for GET disputes, await loading state,
  remove emoji assertion from header
- Host dashboard: accept #9CA3AF badge color for DRAFT status

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documentation/Issue-tracker-spotzy.xlsx
+++ b/documentation/Issue-tracker-spotzy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/orfeopreto/Dev/Claude/spotzy/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2A3C5EF-419A-4D48-85F3-5B7606C16A4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BE67998-A5E4-5E48-AF2C-034505FF0691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="1" xr2:uid="{EF712131-2427-7943-B2E8-AD061EC4DE1A}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Sheet1 (2)" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sheet1 (2)'!$A$1:$G$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sheet1 (2)'!$A$1:$G$57</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="162">
   <si>
     <t>Host Dashboard</t>
   </si>
@@ -491,6 +491,45 @@
   </si>
   <si>
     <t>should see all messages in previous conversation</t>
+  </si>
+  <si>
+    <t>not saved</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no photo shown </t>
+  </si>
+  <si>
+    <t>dead link</t>
+  </si>
+  <si>
+    <t>should be only for spotter</t>
+  </si>
+  <si>
+    <t>no photo shown</t>
+  </si>
+  <si>
+    <t>public page</t>
+  </si>
+  <si>
+    <t>photo of listing is shown</t>
+  </si>
+  <si>
+    <t>no info of user shown</t>
+  </si>
+  <si>
+    <t>basic user info shown (description)</t>
+  </si>
+  <si>
+    <t>Invoicing details are not saved</t>
+  </si>
+  <si>
+    <t xml:space="preserve">should be saved in dynamodb </t>
+  </si>
+  <si>
+    <t>link to conversation partner redirects to landing page</t>
+  </si>
+  <si>
+    <t>should link to public profile of conversation partner</t>
   </si>
 </sst>
 </file>
@@ -624,7 +663,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -668,6 +707,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2019,7 +2062,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2459A4F-4D1F-D947-9C74-71F227501814}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="47.1640625" customWidth="1"/>
@@ -2027,9 +2070,10 @@
     <col min="4" max="4" width="56.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.33203125" style="1" customWidth="1"/>
     <col min="6" max="6" width="23.83203125" customWidth="1"/>
+    <col min="8" max="8" width="21.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>95</v>
       </c>
@@ -2052,7 +2096,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>9</v>
       </c>
@@ -2072,7 +2116,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>10</v>
       </c>
@@ -2086,10 +2130,13 @@
         <v>23</v>
       </c>
       <c r="F3" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+      <c r="H3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>7</v>
       </c>
@@ -2106,7 +2153,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>17</v>
       </c>
@@ -2126,7 +2173,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>19</v>
       </c>
@@ -2146,7 +2193,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>20</v>
       </c>
@@ -2166,7 +2213,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>21</v>
       </c>
@@ -2186,7 +2233,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>18</v>
       </c>
@@ -2203,7 +2250,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>4</v>
       </c>
@@ -2217,10 +2264,13 @@
         <v>9</v>
       </c>
       <c r="F10" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+      <c r="H10" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>5</v>
       </c>
@@ -2237,7 +2287,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>8</v>
       </c>
@@ -2254,7 +2304,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>11</v>
       </c>
@@ -2274,7 +2324,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>1</v>
       </c>
@@ -2291,7 +2341,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>2</v>
       </c>
@@ -2308,7 +2358,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>3</v>
       </c>
@@ -2325,7 +2375,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>23</v>
       </c>
@@ -2342,7 +2392,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>24</v>
       </c>
@@ -2359,7 +2409,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>26</v>
       </c>
@@ -2373,10 +2423,10 @@
         <v>73</v>
       </c>
       <c r="F19" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>27</v>
       </c>
@@ -2396,7 +2446,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>15</v>
       </c>
@@ -2413,7 +2463,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>12</v>
       </c>
@@ -2433,7 +2483,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>13</v>
       </c>
@@ -2453,7 +2503,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>25</v>
       </c>
@@ -2470,7 +2520,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>22</v>
       </c>
@@ -2487,7 +2537,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>14</v>
       </c>
@@ -2501,10 +2551,13 @@
         <v>39</v>
       </c>
       <c r="F26" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+      <c r="H26" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>31</v>
       </c>
@@ -2521,7 +2574,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>32</v>
       </c>
@@ -2538,7 +2591,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>6</v>
       </c>
@@ -2555,7 +2608,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>33</v>
       </c>
@@ -2575,7 +2628,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>16</v>
       </c>
@@ -2595,7 +2648,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>28</v>
       </c>
@@ -2615,7 +2668,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>29</v>
       </c>
@@ -2635,7 +2688,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>30</v>
       </c>
@@ -2655,7 +2708,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" s="7">
         <v>34</v>
       </c>
@@ -2676,7 +2729,7 @@
       </c>
       <c r="G35" s="7"/>
     </row>
-    <row r="36" spans="1:7" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:8" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" s="8">
         <v>35</v>
       </c>
@@ -2697,7 +2750,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:8" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" s="7">
         <v>36</v>
       </c>
@@ -2714,13 +2767,16 @@
         <v>100</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="G37" s="7">
         <v>33</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="H37" s="19" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A38" s="8">
         <v>37</v>
       </c>
@@ -2741,7 +2797,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:8" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" s="7">
         <v>38</v>
       </c>
@@ -2762,7 +2818,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" s="8">
         <v>39</v>
       </c>
@@ -2785,7 +2841,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="68" hidden="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" s="7">
         <v>40</v>
       </c>
@@ -2806,7 +2862,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:8" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" s="8">
         <v>41</v>
       </c>
@@ -2825,7 +2881,7 @@
       </c>
       <c r="G42" s="8"/>
     </row>
-    <row r="43" spans="1:7" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:8" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" s="7">
         <v>42</v>
       </c>
@@ -2844,7 +2900,7 @@
       </c>
       <c r="G43" s="7"/>
     </row>
-    <row r="44" spans="1:7" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:8" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" s="8">
         <v>43</v>
       </c>
@@ -2865,7 +2921,7 @@
       </c>
       <c r="G44" s="8"/>
     </row>
-    <row r="45" spans="1:7" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A45" s="9">
         <v>44</v>
       </c>
@@ -2886,7 +2942,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46" s="18">
         <v>45</v>
       </c>
@@ -2899,11 +2955,14 @@
       <c r="E46" s="1" t="s">
         <v>131</v>
       </c>
+      <c r="F46" s="23" t="s">
+        <v>96</v>
+      </c>
       <c r="G46">
         <v>24</v>
       </c>
     </row>
-    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" s="19">
         <v>46</v>
       </c>
@@ -2923,7 +2982,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A48" s="18">
         <v>47</v>
       </c>
@@ -2963,7 +3022,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:7" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50" s="18">
         <v>49</v>
       </c>
@@ -2975,6 +3034,9 @@
       </c>
       <c r="E50" s="1" t="s">
         <v>139</v>
+      </c>
+      <c r="F50" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="34" x14ac:dyDescent="0.2">
@@ -2987,11 +3049,14 @@
       <c r="E51" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="F51" t="s">
+        <v>96</v>
+      </c>
       <c r="G51">
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:7" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="C52" s="22" t="s">
         <v>145</v>
       </c>
@@ -3000,6 +3065,9 @@
       </c>
       <c r="E52" s="1" t="s">
         <v>73</v>
+      </c>
+      <c r="F52" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="34" x14ac:dyDescent="0.2">
@@ -3018,10 +3086,56 @@
       <c r="E53" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="F53" s="8"/>
+      <c r="F53" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="C54" s="24" t="s">
+        <v>153</v>
+      </c>
+      <c r="D54" s="23" t="s">
+        <v>155</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="C55" s="24" t="s">
+        <v>156</v>
+      </c>
+      <c r="D55" s="23" t="s">
+        <v>157</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="C56" s="24" t="s">
+        <v>158</v>
+      </c>
+      <c r="D56" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="C57" s="24" t="s">
+        <v>160</v>
+      </c>
+      <c r="D57" s="23" t="s">
+        <v>161</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G53" xr:uid="{E2459A4F-4D1F-D947-9C74-71F227501814}">
+  <autoFilter ref="A1:G57" xr:uid="{E2459A4F-4D1F-D947-9C74-71F227501814}">
     <filterColumn colId="5">
       <filters blank="1">
         <filter val="no"/>

</xml_diff>

<commit_message>
UAT Round 5 — fix 14 persistent + new issues
- Spotter dashboard: deriveBookingStatus (CONFIRMED→ACTIVE/COMPLETED)
- ModifyModal: pricePerHour calculated from startTime/endTime (not startDate/endDate)
- Booking interface: added pricePerHour field
- Search dropdown: delayed blur (200ms) so onMouseDown can register
- SpotSummaryCard: price on separate line from rating/distance
- Chat container: calc(100vh - 120px) for proper navbar clearance
- Invoicing section: hidden for non-hosts on profile page
- Public profile: safe photo extraction (handles string and object formats)
- Map popup: dynamic width based on map container (40% max)
- Cancel button: hidden for ACTIVE bookings on spotter dashboard

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documentation/Issue-tracker-spotzy.xlsx
+++ b/documentation/Issue-tracker-spotzy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/orfeopreto/Dev/Claude/spotzy/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A92F97D7-B3FA-324C-8ECF-14933D42E472}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34387AC6-A92C-3547-B13C-77317D4421BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="1" xr2:uid="{EF712131-2427-7943-B2E8-AD061EC4DE1A}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="176">
   <si>
     <t>Host Dashboard</t>
   </si>
@@ -475,9 +475,6 @@
     <t>redirect to listing edit page</t>
   </si>
   <si>
-    <t>chat window height is 20% but the container size is still too big</t>
-  </si>
-  <si>
     <t>cointainer of chat window must be resized too (20% of screen height)</t>
   </si>
   <si>
@@ -530,6 +527,54 @@
   </si>
   <si>
     <t>should link to public profile of conversation partner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">invoicing details are shown on spotter profile </t>
+  </si>
+  <si>
+    <t>should not be shown for non-hosts</t>
+  </si>
+  <si>
+    <t>height of both chat window and its container is too big.
+Cannot see header navbar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">advancing end time one hour </t>
+  </si>
+  <si>
+    <t xml:space="preserve">total refund incorrectly shown but on submit the correct refund was applied
+</t>
+  </si>
+  <si>
+    <t>correct refund (for one hour) should be shown and applied</t>
+  </si>
+  <si>
+    <t xml:space="preserve">advancing start time one hour </t>
+  </si>
+  <si>
+    <t xml:space="preserve">total extra cost incorrectly shown but on submit the correct extra cost was applied
+</t>
+  </si>
+  <si>
+    <t>correct extra cost (for one hour) should be shown and applied</t>
+  </si>
+  <si>
+    <t>status badge showing confirmed iso active</t>
+  </si>
+  <si>
+    <t>should be active</t>
+  </si>
+  <si>
+    <t>booking dashboard</t>
+  </si>
+  <si>
+    <t>s</t>
+  </si>
+  <si>
+    <t>start time is changeable and gets refunded</t>
+  </si>
+  <si>
+    <t xml:space="preserve">line breaks after price </t>
   </si>
 </sst>
 </file>
@@ -2062,7 +2107,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2459A4F-4D1F-D947-9C74-71F227501814}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="47.1640625" customWidth="1"/>
@@ -2133,7 +2178,7 @@
         <v>106</v>
       </c>
       <c r="H3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
@@ -2190,7 +2235,7 @@
         <v>56</v>
       </c>
       <c r="F6" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -2210,7 +2255,7 @@
         <v>56</v>
       </c>
       <c r="F7" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
@@ -2230,7 +2275,7 @@
         <v>56</v>
       </c>
       <c r="F8" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
@@ -2247,7 +2292,7 @@
         <v>52</v>
       </c>
       <c r="F9" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
@@ -2267,7 +2312,7 @@
         <v>106</v>
       </c>
       <c r="H10" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
@@ -2471,7 +2516,7 @@
         <v>30</v>
       </c>
       <c r="C22" t="s">
-        <v>31</v>
+        <v>174</v>
       </c>
       <c r="D22" t="s">
         <v>32</v>
@@ -2500,7 +2545,7 @@
         <v>33</v>
       </c>
       <c r="F23" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
     </row>
     <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
@@ -2554,7 +2599,7 @@
         <v>106</v>
       </c>
       <c r="H26" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
@@ -2699,7 +2744,7 @@
         <v>82</v>
       </c>
       <c r="D34" t="s">
-        <v>83</v>
+        <v>175</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>46</v>
@@ -2773,7 +2818,7 @@
         <v>33</v>
       </c>
       <c r="H37" s="19" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="17" x14ac:dyDescent="0.2">
@@ -2956,7 +3001,7 @@
         <v>131</v>
       </c>
       <c r="F46" s="23" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="G46">
         <v>24</v>
@@ -3041,10 +3086,10 @@
     </row>
     <row r="51" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="C51" s="22" t="s">
+        <v>163</v>
+      </c>
+      <c r="D51" t="s">
         <v>143</v>
-      </c>
-      <c r="D51" t="s">
-        <v>144</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>9</v>
@@ -3058,10 +3103,10 @@
     </row>
     <row r="52" spans="1:7" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="C52" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="D52" t="s">
         <v>145</v>
-      </c>
-      <c r="D52" t="s">
-        <v>146</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>73</v>
@@ -3078,10 +3123,10 @@
         <v>112</v>
       </c>
       <c r="C53" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="D53" s="8" t="s">
         <v>147</v>
-      </c>
-      <c r="D53" s="8" t="s">
-        <v>148</v>
       </c>
       <c r="E53" s="15" t="s">
         <v>115</v>
@@ -3092,46 +3137,119 @@
     </row>
     <row r="54" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="C54" s="24" t="s">
+        <v>152</v>
+      </c>
+      <c r="D54" s="23" t="s">
+        <v>154</v>
+      </c>
+      <c r="E54" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="D54" s="23" t="s">
-        <v>155</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>154</v>
+      <c r="F54" s="23" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="C55" s="24" t="s">
+        <v>155</v>
+      </c>
+      <c r="D55" s="23" t="s">
         <v>156</v>
       </c>
-      <c r="D55" s="23" t="s">
-        <v>157</v>
-      </c>
       <c r="E55" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
+      </c>
+      <c r="F55" s="23" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="C56" s="24" t="s">
+        <v>157</v>
+      </c>
+      <c r="D56" s="23" t="s">
         <v>158</v>
-      </c>
-      <c r="D56" s="23" t="s">
-        <v>159</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="F56" s="23" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="57" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="C57" s="24" t="s">
+        <v>159</v>
+      </c>
+      <c r="D57" s="23" t="s">
         <v>160</v>
-      </c>
-      <c r="D57" s="23" t="s">
-        <v>161</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>9</v>
+      </c>
+      <c r="F57" s="23" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="C58" s="24" t="s">
+        <v>161</v>
+      </c>
+      <c r="D58" s="23" t="s">
+        <v>162</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="B59" s="24" t="s">
+        <v>164</v>
+      </c>
+      <c r="C59" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="D59" s="23" t="s">
+        <v>166</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="B60" s="24" t="s">
+        <v>167</v>
+      </c>
+      <c r="C60" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="D60" s="23" t="s">
+        <v>169</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="B61" t="s">
+        <v>34</v>
+      </c>
+      <c r="C61" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="D61" s="23" t="s">
+        <v>171</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="B62" t="s">
+        <v>34</v>
+      </c>
+      <c r="C62" s="11" t="s">
+        <v>173</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sessions 19-20, UAT2 fixes, backoffice, dev-local environment
- Session 19: User identity (pseudo/display name, profile photo, UserAvatar)
- Session 20: Backoffice (admin guard, disputes dashboard, customer list/detail, AI escalation summary)
- UAT2 fixes: review editing window, dispute bot escalation, customer data, routing
- Dev-local environment: isolated localhost backend (DynamoDB, Cognito, API Gateway)
- Hourly booking status cleanup Lambda
- Documentation updates (v8 specs, archived old versions)
- Add .env.test to .gitignore

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documentation/Issue-tracker-spotzy.xlsx
+++ b/documentation/Issue-tracker-spotzy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/orfeopreto/Dev/Claude/spotzy/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{242FA074-BAFE-484E-BE5A-63260533FB5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7671C22D-7671-0240-B14A-C482F9C5EC6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="640" windowWidth="30240" windowHeight="18280" activeTab="1" xr2:uid="{EF712131-2427-7943-B2E8-AD061EC4DE1A}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="220">
   <si>
     <t>Host Dashboard</t>
   </si>
@@ -674,13 +674,49 @@
     <t xml:space="preserve"> when clicking on submit rating </t>
   </si>
   <si>
-    <t>dispute agent has no access to uploaded images</t>
-  </si>
-  <si>
-    <t>should access uploaded image to either process or pass on to human agent.</t>
-  </si>
-  <si>
     <t>pop up disappears and rating is applied</t>
+  </si>
+  <si>
+    <t>clicking on leave review. Booking already rated.</t>
+  </si>
+  <si>
+    <t>Previous review not shown. Possible to vote.
+on "Submit Rating" error message appears "You have already reviewed this booking"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Previous votes are shown but are editable for 48h.
+On "Submit Rating" new review is applied.
+Beyond 48h voting disabled and submit button disabled.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dispute bot doesn't escalate </t>
+  </si>
+  <si>
+    <t>dispute bot cannot help directly</t>
+  </si>
+  <si>
+    <t>should escalate to admin. Escalation is visible on disputes page in backoffice</t>
+  </si>
+  <si>
+    <t>/backoffice/customers</t>
+  </si>
+  <si>
+    <t>Name always filled in, Rating filled in if exists, Listings and booking show correct values</t>
+  </si>
+  <si>
+    <t>rows for all customers are shown but no fields are empty.
+Exception: Personas (all ok) and Name (only one row with a value in name field)
+Listings and bookings show 0 for all although bookings and listings exist</t>
+  </si>
+  <si>
+    <t>clicking on customer name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">redirected to landing page (probably 404) </t>
+  </si>
+  <si>
+    <t>redirected to customer's profile</t>
   </si>
 </sst>
 </file>
@@ -2225,7 +2261,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2459A4F-4D1F-D947-9C74-71F227501814}">
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="47.1640625" customWidth="1"/>
@@ -3628,31 +3664,67 @@
         <v>205</v>
       </c>
       <c r="D73" s="11" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="E73" s="1" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="74" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A74">
-        <v>72</v>
+      <c r="F73" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+      <c r="B74" t="s">
+        <v>208</v>
       </c>
       <c r="C74" s="11" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D74" s="11" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="E74" s="1" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="B75" t="s">
+        <v>212</v>
+      </c>
+      <c r="C75" s="11" t="s">
+        <v>211</v>
+      </c>
+      <c r="D75" s="11" t="s">
+        <v>213</v>
+      </c>
+      <c r="E75" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A75">
-        <v>73</v>
-      </c>
-      <c r="C75" s="11"/>
+    <row r="76" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+      <c r="C76" s="11" t="s">
+        <v>216</v>
+      </c>
+      <c r="D76" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="E76" s="1" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="B77" t="s">
+        <v>217</v>
+      </c>
+      <c r="C77" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="D77" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="E77" s="1" t="s">
+        <v>214</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H72" xr:uid="{E2459A4F-4D1F-D947-9C74-71F227501814}">

</xml_diff>

<commit_message>
Polish: host landing fixes, nl-BE translations, invoicing required, CORS deployed
- Fix duplicate nav on landing: hide app-shell nav/footer on landing route
- Fix i18n: rebuild translation JSON bundles from YAML, fix duplicate YAML keys
- Add nl-BE translations for all Session 31 host landing keys
- Hero subtitle: improve contrast (#6EE7A0), force white title
- Nav CTA: prevent text wrap with whitespace-nowrap + flex-shrink-0
- Invoicing: billing address required, company name optional, remove skip button
- Register: prefill firstName/lastName/email from landing form query params
- Spotter landing available at /{locale}/spotter
- Add NEXT_PUBLIC_LAUNCH_MODE=prelaunch to .env.local

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documentation/Issue-tracker-spotzy.xlsx
+++ b/documentation/Issue-tracker-spotzy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/orfeopreto/Dev/Claude/spotzy/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{540ABA36-6AE2-CE4E-98F4-77D0F1125534}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DB988E0-E190-6548-8AAA-24A40CF3D6E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="640" windowWidth="30240" windowHeight="18280" activeTab="1" xr2:uid="{EF712131-2427-7943-B2E8-AD061EC4DE1A}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="229">
   <si>
     <t>Host Dashboard</t>
   </si>
@@ -719,33 +719,31 @@
     <t>redirected to customer's profile</t>
   </si>
   <si>
-    <t>apply by day/week/month prices</t>
-  </si>
-  <si>
-    <t>smart tarifs</t>
-  </si>
-  <si>
-    <t>toggle ev (no = red)</t>
-  </si>
-  <si>
-    <t>magic link on arrival; deletion 48h after end of booking</t>
-  </si>
-  <si>
-    <t xml:space="preserve">step 5 allocation </t>
-  </si>
-  <si>
-    <t>hole 7 guests</t>
-  </si>
-  <si>
-    <t>first fill individual spots (no shows more expensive)</t>
-  </si>
-  <si>
-    <t>hole 6</t>
-  </si>
-  <si>
-    <t>1. capture floor on booking day
-2. authorize rest on booking start
-3. booking may not exceed 7 days</t>
+    <t>filter with past start date</t>
+  </si>
+  <si>
+    <t>possible to specify past date</t>
+  </si>
+  <si>
+    <t>not possible to specify past date (should be disabled in control on search page)</t>
+  </si>
+  <si>
+    <t>general</t>
+  </si>
+  <si>
+    <t>validation error occured</t>
+  </si>
+  <si>
+    <t>error is shown in json format</t>
+  </si>
+  <si>
+    <t>error is shown in user friendly format</t>
+  </si>
+  <si>
+    <t>avaiilability filter has no effect</t>
+  </si>
+  <si>
+    <t>filters on selected criteria</t>
   </si>
 </sst>
 </file>
@@ -2291,12 +2289,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2459A4F-4D1F-D947-9C74-71F227501814}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:H86"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="47.1640625" customWidth="1"/>
     <col min="3" max="3" width="50.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="56.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="67" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.33203125" style="1" customWidth="1"/>
     <col min="6" max="6" width="23.83203125" customWidth="1"/>
     <col min="8" max="8" width="21.6640625" bestFit="1" customWidth="1"/>
@@ -3609,7 +3607,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="69" spans="1:7" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:7" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>67</v>
       </c>
@@ -3720,7 +3718,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="75" spans="1:7" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:7" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="B75" t="s">
         <v>212</v>
       </c>
@@ -3768,52 +3766,49 @@
         <v>106</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="D78" t="s">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B79" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="C79" t="s">
+        <v>221</v>
+      </c>
       <c r="D79" t="s">
-        <v>221</v>
+        <v>222</v>
+      </c>
+      <c r="E79" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="F79" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B80" t="s">
+        <v>224</v>
+      </c>
+      <c r="C80" t="s">
+        <v>225</v>
+      </c>
       <c r="D80" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="82" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C82">
-        <v>1444</v>
-      </c>
-      <c r="D82">
-        <f>C82*0.2</f>
-        <v>288.8</v>
-      </c>
-    </row>
-    <row r="84" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B84" t="s">
-        <v>225</v>
-      </c>
-      <c r="D84" t="s">
+        <v>226</v>
+      </c>
+      <c r="E80" s="1" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="85" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B85" t="s">
-        <v>224</v>
-      </c>
-      <c r="D85" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="86" spans="2:4" ht="51" x14ac:dyDescent="0.2">
-      <c r="B86" t="s">
+    <row r="81" spans="3:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="C81" t="s">
         <v>227</v>
       </c>
-      <c r="D86" s="11" t="s">
+      <c r="D81" s="11" t="s">
         <v>228</v>
+      </c>
+      <c r="E81" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="F81" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>